<commit_message>
📦 Added DSC, Mill Return, and Reporting Month files
</commit_message>
<xml_diff>
--- a/data/tractor_operations.xlsx
+++ b/data/tractor_operations.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Date</t>
   </si>
@@ -58,102 +58,6 @@
   </si>
   <si>
     <t>Season</t>
-  </si>
-  <si>
-    <t>2025-3-1</t>
-  </si>
-  <si>
-    <t>BU892</t>
-  </si>
-  <si>
-    <t>Jimmy Mack</t>
-  </si>
-  <si>
-    <t>DG010001</t>
-  </si>
-  <si>
-    <t>Banking</t>
-  </si>
-  <si>
-    <t>2025/26</t>
-  </si>
-  <si>
-    <t>2024-9-22</t>
-  </si>
-  <si>
-    <t>KK12</t>
-  </si>
-  <si>
-    <t>January</t>
-  </si>
-  <si>
-    <t>DG4</t>
-  </si>
-  <si>
-    <t>Harrow</t>
-  </si>
-  <si>
-    <t>2025-4-1</t>
-  </si>
-  <si>
-    <t>Palanjenta</t>
-  </si>
-  <si>
-    <t>LF06005</t>
-  </si>
-  <si>
-    <t>Fertilizer delivary</t>
-  </si>
-  <si>
-    <t>2025-06-05</t>
-  </si>
-  <si>
-    <t>BR4582</t>
-  </si>
-  <si>
-    <t>P Sibale</t>
-  </si>
-  <si>
-    <t>DG11000</t>
-  </si>
-  <si>
-    <t>DG25006</t>
-  </si>
-  <si>
-    <t>Harrowing</t>
-  </si>
-  <si>
-    <t>2025-06-03</t>
-  </si>
-  <si>
-    <t>KK1049</t>
-  </si>
-  <si>
-    <t>C January</t>
-  </si>
-  <si>
-    <t>LP05005</t>
-  </si>
-  <si>
-    <t>Rigging</t>
-  </si>
-  <si>
-    <t>New plant</t>
-  </si>
-  <si>
-    <t>BU900</t>
-  </si>
-  <si>
-    <t>Itimu</t>
-  </si>
-  <si>
-    <t>DG16000</t>
-  </si>
-  <si>
-    <t>Ripping</t>
-  </si>
-  <si>
-    <t>Dry Field</t>
   </si>
   <si>
     <t>Area (ha)</t>
@@ -519,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -566,7 +470,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>9</v>
@@ -579,266 +483,6 @@
       </c>
       <c r="N1" s="1" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2">
-        <v>1234</v>
-      </c>
-      <c r="G2">
-        <v>1238</v>
-      </c>
-      <c r="I2">
-        <v>15</v>
-      </c>
-      <c r="J2">
-        <v>3</v>
-      </c>
-      <c r="N2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3">
-        <v>1234</v>
-      </c>
-      <c r="G3">
-        <v>1236</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>10</v>
-      </c>
-      <c r="J3">
-        <v>3</v>
-      </c>
-      <c r="N3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4">
-        <v>111049</v>
-      </c>
-      <c r="G4">
-        <v>111063</v>
-      </c>
-      <c r="H4">
-        <v>14</v>
-      </c>
-      <c r="I4">
-        <v>35</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="N4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5">
-        <v>1234.8</v>
-      </c>
-      <c r="G5">
-        <v>1268.5</v>
-      </c>
-      <c r="H5">
-        <v>33.700000000000003</v>
-      </c>
-      <c r="I5">
-        <v>25</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="N5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6">
-        <v>1049.3</v>
-      </c>
-      <c r="G6">
-        <v>1052.8</v>
-      </c>
-      <c r="H6">
-        <v>3.5</v>
-      </c>
-      <c r="I6">
-        <v>31</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="N6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>35</v>
-      </c>
-      <c r="J7">
-        <v>1.89</v>
-      </c>
-      <c r="K7">
-        <v>18.52</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7" t="s">
-        <v>39</v>
-      </c>
-      <c r="N7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8">
-        <v>700.8</v>
-      </c>
-      <c r="G8">
-        <v>712.3</v>
-      </c>
-      <c r="H8">
-        <v>11.5</v>
-      </c>
-      <c r="I8">
-        <v>35.799999999999997</v>
-      </c>
-      <c r="J8">
-        <v>4.8600000000000003</v>
-      </c>
-      <c r="K8">
-        <v>7.37</v>
-      </c>
-      <c r="L8">
-        <v>2.37</v>
-      </c>
-      <c r="M8" t="s">
-        <v>44</v>
-      </c>
-      <c r="N8" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>